<commit_message>
Atualização com coluna Bloqueado
</commit_message>
<xml_diff>
--- a/Base_Consolidada_SIAFI.xlsx
+++ b/Base_Consolidada_SIAFI.xlsx
@@ -63999,7 +63999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z130"/>
+  <dimension ref="A1:AC130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -64120,15 +64120,30 @@
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
+          <t>Bloqueado_Ant</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Bloqueado_Atual</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>Variação_Bloqueado</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
           <t>Disponível_Ant</t>
         </is>
       </c>
-      <c r="Y1" s="1" t="inlineStr">
+      <c r="AB1" s="1" t="inlineStr">
         <is>
           <t>Disponível_Atual</t>
         </is>
       </c>
-      <c r="Z1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>Variação_Disponível</t>
         </is>
@@ -64211,12 +64226,21 @@
         <v>0</v>
       </c>
       <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z2" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA2" t="n">
         <v>1072500</v>
       </c>
-      <c r="Y2" t="n">
+      <c r="AB2" t="n">
         <v>1072500</v>
       </c>
-      <c r="Z2" t="n">
+      <c r="AC2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -64297,12 +64321,21 @@
         <v>526440</v>
       </c>
       <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA3" t="n">
         <v>12300</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="AB3" t="n">
         <v>12300</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AC3" t="n">
         <v>0</v>
       </c>
     </row>
@@ -64383,12 +64416,21 @@
         <v>0</v>
       </c>
       <c r="X4" t="n">
+        <v>150000</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>150000</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA4" t="n">
         <v>97412</v>
       </c>
-      <c r="Y4" t="n">
+      <c r="AB4" t="n">
         <v>97412</v>
       </c>
-      <c r="Z4" t="n">
+      <c r="AC4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -64469,12 +64511,21 @@
         <v>20000</v>
       </c>
       <c r="X5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z5" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA5" t="n">
         <v>485000</v>
       </c>
-      <c r="Y5" t="n">
+      <c r="AB5" t="n">
         <v>485000</v>
       </c>
-      <c r="Z5" t="n">
+      <c r="AC5" t="n">
         <v>0</v>
       </c>
     </row>
@@ -64555,12 +64606,21 @@
         <v>281744.6</v>
       </c>
       <c r="X6" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="Y6" t="n">
+        <v>1500000</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA6" t="n">
         <v>2594035.9</v>
       </c>
-      <c r="Y6" t="n">
+      <c r="AB6" t="n">
         <v>2594035.9</v>
       </c>
-      <c r="Z6" t="n">
+      <c r="AC6" t="n">
         <v>0</v>
       </c>
     </row>
@@ -64649,6 +64709,15 @@
       <c r="Z7" t="n">
         <v>0</v>
       </c>
+      <c r="AA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB7" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -64727,12 +64796,21 @@
         <v>0</v>
       </c>
       <c r="X8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z8" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA8" t="n">
         <v>15770</v>
       </c>
-      <c r="Y8" t="n">
+      <c r="AB8" t="n">
         <v>15770</v>
       </c>
-      <c r="Z8" t="n">
+      <c r="AC8" t="n">
         <v>0</v>
       </c>
     </row>
@@ -64813,12 +64891,21 @@
         <v>1329599.219999999</v>
       </c>
       <c r="X9" t="n">
+        <v>46382823.26</v>
+      </c>
+      <c r="Y9" t="n">
+        <v>52882823.26</v>
+      </c>
+      <c r="Z9" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="AA9" t="n">
         <v>19401015.72</v>
       </c>
-      <c r="Y9" t="n">
+      <c r="AB9" t="n">
         <v>12901015.72</v>
       </c>
-      <c r="Z9" t="n">
+      <c r="AC9" t="n">
         <v>-6499999.999999998</v>
       </c>
     </row>
@@ -64899,12 +64986,21 @@
         <v>1462988.71</v>
       </c>
       <c r="X10" t="n">
+        <v>27222950.51</v>
+      </c>
+      <c r="Y10" t="n">
+        <v>28888082.39</v>
+      </c>
+      <c r="Z10" t="n">
+        <v>1665131.879999999</v>
+      </c>
+      <c r="AA10" t="n">
         <v>21872955.56</v>
       </c>
-      <c r="Y10" t="n">
+      <c r="AB10" t="n">
         <v>20207823.68</v>
       </c>
-      <c r="Z10" t="n">
+      <c r="AC10" t="n">
         <v>-1665131.879999999</v>
       </c>
     </row>
@@ -64985,12 +65081,21 @@
         <v>5389734.240000002</v>
       </c>
       <c r="X11" t="n">
+        <v>46897827.05</v>
+      </c>
+      <c r="Y11" t="n">
+        <v>53397827.05</v>
+      </c>
+      <c r="Z11" t="n">
+        <v>6500000</v>
+      </c>
+      <c r="AA11" t="n">
         <v>27724491.19</v>
       </c>
-      <c r="Y11" t="n">
+      <c r="AB11" t="n">
         <v>18646285.19</v>
       </c>
-      <c r="Z11" t="n">
+      <c r="AC11" t="n">
         <v>-9078206</v>
       </c>
     </row>
@@ -65071,12 +65176,21 @@
         <v>1080</v>
       </c>
       <c r="X12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y12" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z12" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA12" t="n">
         <v>2712344.4</v>
       </c>
-      <c r="Y12" t="n">
+      <c r="AB12" t="n">
         <v>2696107.6</v>
       </c>
-      <c r="Z12" t="n">
+      <c r="AC12" t="n">
         <v>-16236.79999999981</v>
       </c>
     </row>
@@ -65157,12 +65271,21 @@
         <v>2593798.539999999</v>
       </c>
       <c r="X13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y13" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z13" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA13" t="n">
         <v>1045530.35</v>
       </c>
-      <c r="Y13" t="n">
+      <c r="AB13" t="n">
         <v>3623736.35</v>
       </c>
-      <c r="Z13" t="n">
+      <c r="AC13" t="n">
         <v>2578206</v>
       </c>
     </row>
@@ -65243,12 +65366,21 @@
         <v>864915.1199999999</v>
       </c>
       <c r="X14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y14" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z14" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA14" t="n">
         <v>10102333.08</v>
       </c>
-      <c r="Y14" t="n">
+      <c r="AB14" t="n">
         <v>8763041.26</v>
       </c>
-      <c r="Z14" t="n">
+      <c r="AC14" t="n">
         <v>-1339291.82</v>
       </c>
     </row>
@@ -65329,12 +65461,21 @@
         <v>0</v>
       </c>
       <c r="X15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y15" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z15" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA15" t="n">
         <v>1650000</v>
       </c>
-      <c r="Y15" t="n">
+      <c r="AB15" t="n">
         <v>1650000</v>
       </c>
-      <c r="Z15" t="n">
+      <c r="AC15" t="n">
         <v>0</v>
       </c>
     </row>
@@ -65415,12 +65556,21 @@
         <v>73024</v>
       </c>
       <c r="X16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y16" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z16" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA16" t="n">
         <v>1932326</v>
       </c>
-      <c r="Y16" t="n">
+      <c r="AB16" t="n">
         <v>1932326</v>
       </c>
-      <c r="Z16" t="n">
+      <c r="AC16" t="n">
         <v>0</v>
       </c>
     </row>
@@ -65501,12 +65651,21 @@
         <v>396970.3500000006</v>
       </c>
       <c r="X17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y17" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z17" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA17" t="n">
         <v>22791039.49</v>
       </c>
-      <c r="Y17" t="n">
+      <c r="AB17" t="n">
         <v>24164795.07</v>
       </c>
-      <c r="Z17" t="n">
+      <c r="AC17" t="n">
         <v>1373755.580000002</v>
       </c>
     </row>
@@ -65587,12 +65746,21 @@
         <v>14714.66</v>
       </c>
       <c r="X18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y18" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z18" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA18" t="n">
         <v>105856.02</v>
       </c>
-      <c r="Y18" t="n">
+      <c r="AB18" t="n">
         <v>105856.02</v>
       </c>
-      <c r="Z18" t="n">
+      <c r="AC18" t="n">
         <v>0</v>
       </c>
     </row>
@@ -65673,12 +65841,21 @@
         <v>8395377.629999995</v>
       </c>
       <c r="X19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y19" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z19" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA19" t="n">
         <v>278444787.27</v>
       </c>
-      <c r="Y19" t="n">
+      <c r="AB19" t="n">
         <v>278449528.26</v>
       </c>
-      <c r="Z19" t="n">
+      <c r="AC19" t="n">
         <v>4740.990000009537</v>
       </c>
     </row>
@@ -65759,12 +65936,21 @@
         <v>213.5100000000093</v>
       </c>
       <c r="X20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y20" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z20" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA20" t="n">
         <v>3530858.84</v>
       </c>
-      <c r="Y20" t="n">
+      <c r="AB20" t="n">
         <v>3544564.98</v>
       </c>
-      <c r="Z20" t="n">
+      <c r="AC20" t="n">
         <v>13706.14000000013</v>
       </c>
     </row>
@@ -65853,6 +66039,15 @@
       <c r="Z21" t="n">
         <v>0</v>
       </c>
+      <c r="AA21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -65931,12 +66126,21 @@
         <v>0</v>
       </c>
       <c r="X22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="n">
         <v>139.09</v>
       </c>
-      <c r="Y22" t="n">
+      <c r="AB22" t="n">
         <v>139.09</v>
       </c>
-      <c r="Z22" t="n">
+      <c r="AC22" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66017,12 +66221,21 @@
         <v>3113406.819999999</v>
       </c>
       <c r="X23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="n">
         <v>30895406.07</v>
       </c>
-      <c r="Y23" t="n">
+      <c r="AB23" t="n">
         <v>30895406.07</v>
       </c>
-      <c r="Z23" t="n">
+      <c r="AC23" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66103,12 +66316,21 @@
         <v>0</v>
       </c>
       <c r="X24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA24" t="n">
         <v>6594301</v>
       </c>
-      <c r="Y24" t="n">
+      <c r="AB24" t="n">
         <v>6594301</v>
       </c>
-      <c r="Z24" t="n">
+      <c r="AC24" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66189,12 +66411,21 @@
         <v>0</v>
       </c>
       <c r="X25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z25" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA25" t="n">
         <v>9332401.09</v>
       </c>
-      <c r="Y25" t="n">
+      <c r="AB25" t="n">
         <v>9332401.09</v>
       </c>
-      <c r="Z25" t="n">
+      <c r="AC25" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66275,12 +66506,21 @@
         <v>0</v>
       </c>
       <c r="X26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA26" t="n">
         <v>452205.65</v>
       </c>
-      <c r="Y26" t="n">
+      <c r="AB26" t="n">
         <v>38678.68</v>
       </c>
-      <c r="Z26" t="n">
+      <c r="AC26" t="n">
         <v>-413526.97</v>
       </c>
     </row>
@@ -66361,12 +66601,21 @@
         <v>220812.59</v>
       </c>
       <c r="X27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y27" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z27" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA27" t="n">
         <v>4232604.14</v>
       </c>
-      <c r="Y27" t="n">
+      <c r="AB27" t="n">
         <v>4232604.14</v>
       </c>
-      <c r="Z27" t="n">
+      <c r="AC27" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66447,12 +66696,21 @@
         <v>0</v>
       </c>
       <c r="X28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y28" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z28" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA28" t="n">
         <v>52328.35</v>
       </c>
-      <c r="Y28" t="n">
+      <c r="AB28" t="n">
         <v>29796.8</v>
       </c>
-      <c r="Z28" t="n">
+      <c r="AC28" t="n">
         <v>-22531.55</v>
       </c>
     </row>
@@ -66533,12 +66791,21 @@
         <v>0</v>
       </c>
       <c r="X29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y29" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z29" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA29" t="n">
         <v>4050200</v>
       </c>
-      <c r="Y29" t="n">
+      <c r="AB29" t="n">
         <v>4050200</v>
       </c>
-      <c r="Z29" t="n">
+      <c r="AC29" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66619,12 +66886,21 @@
         <v>0</v>
       </c>
       <c r="X30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y30" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z30" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA30" t="n">
         <v>10000</v>
       </c>
-      <c r="Y30" t="n">
+      <c r="AB30" t="n">
         <v>10000</v>
       </c>
-      <c r="Z30" t="n">
+      <c r="AC30" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66705,12 +66981,21 @@
         <v>0</v>
       </c>
       <c r="X31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y31" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA31" t="n">
         <v>18540000</v>
       </c>
-      <c r="Y31" t="n">
+      <c r="AB31" t="n">
         <v>18540000</v>
       </c>
-      <c r="Z31" t="n">
+      <c r="AC31" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66791,12 +67076,21 @@
         <v>0</v>
       </c>
       <c r="X32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y32" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA32" t="n">
         <v>500000</v>
       </c>
-      <c r="Y32" t="n">
+      <c r="AB32" t="n">
         <v>500000</v>
       </c>
-      <c r="Z32" t="n">
+      <c r="AC32" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66877,12 +67171,21 @@
         <v>0</v>
       </c>
       <c r="X33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y33" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA33" t="n">
         <v>1292593.07</v>
       </c>
-      <c r="Y33" t="n">
+      <c r="AB33" t="n">
         <v>1292593.07</v>
       </c>
-      <c r="Z33" t="n">
+      <c r="AC33" t="n">
         <v>0</v>
       </c>
     </row>
@@ -66963,12 +67266,21 @@
         <v>0</v>
       </c>
       <c r="X34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y34" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z34" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA34" t="n">
         <v>770000</v>
       </c>
-      <c r="Y34" t="n">
+      <c r="AB34" t="n">
         <v>770000</v>
       </c>
-      <c r="Z34" t="n">
+      <c r="AC34" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67049,12 +67361,21 @@
         <v>0</v>
       </c>
       <c r="X35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y35" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z35" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA35" t="n">
         <v>19994</v>
       </c>
-      <c r="Y35" t="n">
+      <c r="AB35" t="n">
         <v>19994</v>
       </c>
-      <c r="Z35" t="n">
+      <c r="AC35" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67135,12 +67456,21 @@
         <v>94956</v>
       </c>
       <c r="X36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y36" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z36" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA36" t="n">
         <v>26109.93</v>
       </c>
-      <c r="Y36" t="n">
+      <c r="AB36" t="n">
         <v>26109.93</v>
       </c>
-      <c r="Z36" t="n">
+      <c r="AC36" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67221,12 +67551,21 @@
         <v>7672.950000000012</v>
       </c>
       <c r="X37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y37" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z37" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA37" t="n">
         <v>16522.65</v>
       </c>
-      <c r="Y37" t="n">
+      <c r="AB37" t="n">
         <v>12310.05</v>
       </c>
-      <c r="Z37" t="n">
+      <c r="AC37" t="n">
         <v>-4212.600000000002</v>
       </c>
     </row>
@@ -67307,12 +67646,21 @@
         <v>0</v>
       </c>
       <c r="X38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y38" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z38" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA38" t="n">
         <v>34114.1</v>
       </c>
-      <c r="Y38" t="n">
+      <c r="AB38" t="n">
         <v>34114.1</v>
       </c>
-      <c r="Z38" t="n">
+      <c r="AC38" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67393,12 +67741,21 @@
         <v>24072</v>
       </c>
       <c r="X39" t="n">
+        <v>400000</v>
+      </c>
+      <c r="Y39" t="n">
+        <v>400000</v>
+      </c>
+      <c r="Z39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA39" t="n">
         <v>215417</v>
       </c>
-      <c r="Y39" t="n">
+      <c r="AB39" t="n">
         <v>215417</v>
       </c>
-      <c r="Z39" t="n">
+      <c r="AC39" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67479,12 +67836,21 @@
         <v>0</v>
       </c>
       <c r="X40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA40" t="n">
         <v>15000</v>
       </c>
-      <c r="Y40" t="n">
+      <c r="AB40" t="n">
         <v>15000</v>
       </c>
-      <c r="Z40" t="n">
+      <c r="AC40" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67565,12 +67931,21 @@
         <v>71015.78000000003</v>
       </c>
       <c r="X41" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="Y41" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="Z41" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA41" t="n">
         <v>3347726.48</v>
       </c>
-      <c r="Y41" t="n">
+      <c r="AB41" t="n">
         <v>3347726.48</v>
       </c>
-      <c r="Z41" t="n">
+      <c r="AC41" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67651,12 +68026,21 @@
         <v>3690</v>
       </c>
       <c r="X42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y42" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z42" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA42" t="n">
         <v>1227731.4</v>
       </c>
-      <c r="Y42" t="n">
+      <c r="AB42" t="n">
         <v>1227731.4</v>
       </c>
-      <c r="Z42" t="n">
+      <c r="AC42" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67737,12 +68121,21 @@
         <v>1284165.8</v>
       </c>
       <c r="X43" t="n">
+        <v>16123051.01</v>
+      </c>
+      <c r="Y43" t="n">
+        <v>16123051.01</v>
+      </c>
+      <c r="Z43" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA43" t="n">
         <v>4591755.2</v>
       </c>
-      <c r="Y43" t="n">
+      <c r="AB43" t="n">
         <v>4591755.2</v>
       </c>
-      <c r="Z43" t="n">
+      <c r="AC43" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67823,12 +68216,21 @@
         <v>1532232.82</v>
       </c>
       <c r="X44" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="Y44" t="n">
+        <v>2000000</v>
+      </c>
+      <c r="Z44" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA44" t="n">
         <v>7404963.76</v>
       </c>
-      <c r="Y44" t="n">
+      <c r="AB44" t="n">
         <v>7404963.76</v>
       </c>
-      <c r="Z44" t="n">
+      <c r="AC44" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67909,12 +68311,21 @@
         <v>635409.45</v>
       </c>
       <c r="X45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y45" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA45" t="n">
         <v>5746333.32</v>
       </c>
-      <c r="Y45" t="n">
+      <c r="AB45" t="n">
         <v>5746333.32</v>
       </c>
-      <c r="Z45" t="n">
+      <c r="AC45" t="n">
         <v>0</v>
       </c>
     </row>
@@ -67995,12 +68406,21 @@
         <v>2221970.44</v>
       </c>
       <c r="X46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y46" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z46" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA46" t="n">
         <v>683844.08</v>
       </c>
-      <c r="Y46" t="n">
+      <c r="AB46" t="n">
         <v>683844.08</v>
       </c>
-      <c r="Z46" t="n">
+      <c r="AC46" t="n">
         <v>0</v>
       </c>
     </row>
@@ -68081,12 +68501,21 @@
         <v>0</v>
       </c>
       <c r="X47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA47" t="n">
         <v>10000</v>
       </c>
-      <c r="Y47" t="n">
+      <c r="AB47" t="n">
         <v>10000</v>
       </c>
-      <c r="Z47" t="n">
+      <c r="AC47" t="n">
         <v>0</v>
       </c>
     </row>
@@ -68167,12 +68596,21 @@
         <v>0</v>
       </c>
       <c r="X48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y48" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z48" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA48" t="n">
         <v>665000</v>
       </c>
-      <c r="Y48" t="n">
+      <c r="AB48" t="n">
         <v>665000</v>
       </c>
-      <c r="Z48" t="n">
+      <c r="AC48" t="n">
         <v>0</v>
       </c>
     </row>
@@ -68261,6 +68699,15 @@
       <c r="Z49" t="n">
         <v>0</v>
       </c>
+      <c r="AA49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB49" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -68347,6 +68794,15 @@
       <c r="Z50" t="n">
         <v>0</v>
       </c>
+      <c r="AA50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB50" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -68425,12 +68881,21 @@
         <v>0</v>
       </c>
       <c r="X51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y51" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z51" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA51" t="n">
         <v>9418</v>
       </c>
-      <c r="Y51" t="n">
+      <c r="AB51" t="n">
         <v>9418</v>
       </c>
-      <c r="Z51" t="n">
+      <c r="AC51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -68511,12 +68976,21 @@
         <v>13841.40000000001</v>
       </c>
       <c r="X52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y52" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z52" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA52" t="n">
         <v>141874.35</v>
       </c>
-      <c r="Y52" t="n">
+      <c r="AB52" t="n">
         <v>122466.3</v>
       </c>
-      <c r="Z52" t="n">
+      <c r="AC52" t="n">
         <v>-19408.05</v>
       </c>
     </row>
@@ -68597,12 +69071,21 @@
         <v>0</v>
       </c>
       <c r="X53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y53" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z53" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA53" t="n">
         <v>135746</v>
       </c>
-      <c r="Y53" t="n">
+      <c r="AB53" t="n">
         <v>127320.8</v>
       </c>
-      <c r="Z53" t="n">
+      <c r="AC53" t="n">
         <v>-8425.199999999997</v>
       </c>
     </row>
@@ -68683,12 +69166,21 @@
         <v>30311.5</v>
       </c>
       <c r="X54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y54" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z54" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA54" t="n">
         <v>26683.3</v>
       </c>
-      <c r="Y54" t="n">
+      <c r="AB54" t="n">
         <v>23333.3</v>
       </c>
-      <c r="Z54" t="n">
+      <c r="AC54" t="n">
         <v>-3350</v>
       </c>
     </row>
@@ -68769,12 +69261,21 @@
         <v>11725</v>
       </c>
       <c r="X55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y55" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z55" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA55" t="n">
         <v>17047.7</v>
       </c>
-      <c r="Y55" t="n">
+      <c r="AB55" t="n">
         <v>17047.7</v>
       </c>
-      <c r="Z55" t="n">
+      <c r="AC55" t="n">
         <v>0</v>
       </c>
     </row>
@@ -68858,9 +69359,18 @@
         <v>0</v>
       </c>
       <c r="Y56" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA56" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB56" t="n">
         <v>5000</v>
       </c>
-      <c r="Z56" t="n">
+      <c r="AC56" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -68941,12 +69451,21 @@
         <v>0</v>
       </c>
       <c r="X57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y57" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z57" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA57" t="n">
         <v>5000</v>
       </c>
-      <c r="Y57" t="n">
+      <c r="AB57" t="n">
         <v>5000</v>
       </c>
-      <c r="Z57" t="n">
+      <c r="AC57" t="n">
         <v>0</v>
       </c>
     </row>
@@ -69027,12 +69546,21 @@
         <v>0</v>
       </c>
       <c r="X58" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y58" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA58" t="n">
         <v>5000</v>
       </c>
-      <c r="Y58" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z58" t="n">
+      <c r="AB58" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC58" t="n">
         <v>-5000</v>
       </c>
     </row>
@@ -69116,9 +69644,18 @@
         <v>0</v>
       </c>
       <c r="Y59" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA59" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB59" t="n">
         <v>5000</v>
       </c>
-      <c r="Z59" t="n">
+      <c r="AC59" t="n">
         <v>5000</v>
       </c>
     </row>
@@ -69199,12 +69736,21 @@
         <v>10000</v>
       </c>
       <c r="X60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y60" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z60" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA60" t="n">
         <v>5000</v>
       </c>
-      <c r="Y60" t="n">
+      <c r="AB60" t="n">
         <v>5000</v>
       </c>
-      <c r="Z60" t="n">
+      <c r="AC60" t="n">
         <v>0</v>
       </c>
     </row>
@@ -69293,6 +69839,15 @@
       <c r="Z61" t="n">
         <v>0</v>
       </c>
+      <c r="AA61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB61" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC61" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -69371,12 +69926,21 @@
         <v>5000</v>
       </c>
       <c r="X62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y62" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z62" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA62" t="n">
         <v>5000</v>
       </c>
-      <c r="Y62" t="n">
+      <c r="AB62" t="n">
         <v>5000</v>
       </c>
-      <c r="Z62" t="n">
+      <c r="AC62" t="n">
         <v>0</v>
       </c>
     </row>
@@ -69465,6 +70029,15 @@
       <c r="Z63" t="n">
         <v>0</v>
       </c>
+      <c r="AA63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB63" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -69551,6 +70124,15 @@
       <c r="Z64" t="n">
         <v>0</v>
       </c>
+      <c r="AA64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB64" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC64" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -69637,6 +70219,15 @@
       <c r="Z65" t="n">
         <v>0</v>
       </c>
+      <c r="AA65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB65" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -69723,6 +70314,15 @@
       <c r="Z66" t="n">
         <v>0</v>
       </c>
+      <c r="AA66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB66" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -69801,12 +70401,21 @@
         <v>0</v>
       </c>
       <c r="X67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y67" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z67" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA67" t="n">
         <v>65296.8</v>
       </c>
-      <c r="Y67" t="n">
+      <c r="AB67" t="n">
         <v>122076.6</v>
       </c>
-      <c r="Z67" t="n">
+      <c r="AC67" t="n">
         <v>56779.8</v>
       </c>
     </row>
@@ -69887,12 +70496,21 @@
         <v>10000</v>
       </c>
       <c r="X68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y68" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z68" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA68" t="n">
         <v>5000</v>
       </c>
-      <c r="Y68" t="n">
+      <c r="AB68" t="n">
         <v>5000</v>
       </c>
-      <c r="Z68" t="n">
+      <c r="AC68" t="n">
         <v>0</v>
       </c>
     </row>
@@ -69973,12 +70591,21 @@
         <v>5000</v>
       </c>
       <c r="X69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y69" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z69" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA69" t="n">
         <v>10000</v>
       </c>
-      <c r="Y69" t="n">
+      <c r="AB69" t="n">
         <v>10000</v>
       </c>
-      <c r="Z69" t="n">
+      <c r="AC69" t="n">
         <v>0</v>
       </c>
     </row>
@@ -70067,6 +70694,15 @@
       <c r="Z70" t="n">
         <v>0</v>
       </c>
+      <c r="AA70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB70" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -70153,6 +70789,15 @@
       <c r="Z71" t="n">
         <v>0</v>
       </c>
+      <c r="AA71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB71" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -70239,6 +70884,15 @@
       <c r="Z72" t="n">
         <v>0</v>
       </c>
+      <c r="AA72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB72" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -70325,6 +70979,15 @@
       <c r="Z73" t="n">
         <v>0</v>
       </c>
+      <c r="AA73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB73" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -70411,6 +71074,15 @@
       <c r="Z74" t="n">
         <v>0</v>
       </c>
+      <c r="AA74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB74" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -70497,6 +71169,15 @@
       <c r="Z75" t="n">
         <v>0</v>
       </c>
+      <c r="AA75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB75" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -70583,6 +71264,15 @@
       <c r="Z76" t="n">
         <v>0</v>
       </c>
+      <c r="AA76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB76" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -70669,6 +71359,15 @@
       <c r="Z77" t="n">
         <v>0</v>
       </c>
+      <c r="AA77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB77" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -70755,6 +71454,15 @@
       <c r="Z78" t="n">
         <v>0</v>
       </c>
+      <c r="AA78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB78" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -70841,6 +71549,15 @@
       <c r="Z79" t="n">
         <v>0</v>
       </c>
+      <c r="AA79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB79" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -70927,6 +71644,15 @@
       <c r="Z80" t="n">
         <v>0</v>
       </c>
+      <c r="AA80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB80" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -71005,12 +71731,21 @@
         <v>0</v>
       </c>
       <c r="X81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y81" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z81" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA81" t="n">
         <v>8368410.56</v>
       </c>
-      <c r="Y81" t="n">
+      <c r="AB81" t="n">
         <v>8368410.56</v>
       </c>
-      <c r="Z81" t="n">
+      <c r="AC81" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71091,12 +71826,21 @@
         <v>0</v>
       </c>
       <c r="X82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y82" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z82" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA82" t="n">
         <v>5000000</v>
       </c>
-      <c r="Y82" t="n">
+      <c r="AB82" t="n">
         <v>5000000</v>
       </c>
-      <c r="Z82" t="n">
+      <c r="AC82" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71177,12 +71921,21 @@
         <v>0</v>
       </c>
       <c r="X83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y83" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z83" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA83" t="n">
         <v>199635.07</v>
       </c>
-      <c r="Y83" t="n">
+      <c r="AB83" t="n">
         <v>199635.07</v>
       </c>
-      <c r="Z83" t="n">
+      <c r="AC83" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71271,6 +72024,15 @@
       <c r="Z84" t="n">
         <v>0</v>
       </c>
+      <c r="AA84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB84" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -71349,12 +72111,21 @@
         <v>0</v>
       </c>
       <c r="X85" t="n">
+        <v>1229488.3</v>
+      </c>
+      <c r="Y85" t="n">
+        <v>1229488.3</v>
+      </c>
+      <c r="Z85" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA85" t="n">
         <v>61458.63</v>
       </c>
-      <c r="Y85" t="n">
+      <c r="AB85" t="n">
         <v>61458.63</v>
       </c>
-      <c r="Z85" t="n">
+      <c r="AC85" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71435,12 +72206,21 @@
         <v>0</v>
       </c>
       <c r="X86" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y86" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z86" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA86" t="n">
         <v>64023.02</v>
       </c>
-      <c r="Y86" t="n">
+      <c r="AB86" t="n">
         <v>64023.02</v>
       </c>
-      <c r="Z86" t="n">
+      <c r="AC86" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71529,6 +72309,15 @@
       <c r="Z87" t="n">
         <v>0</v>
       </c>
+      <c r="AA87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB87" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -71607,12 +72396,21 @@
         <v>0</v>
       </c>
       <c r="X88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y88" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z88" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA88" t="n">
         <v>4695093.84</v>
       </c>
-      <c r="Y88" t="n">
+      <c r="AB88" t="n">
         <v>4695093.84</v>
       </c>
-      <c r="Z88" t="n">
+      <c r="AC88" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71693,12 +72491,21 @@
         <v>0</v>
       </c>
       <c r="X89" t="n">
+        <v>100000</v>
+      </c>
+      <c r="Y89" t="n">
+        <v>100000</v>
+      </c>
+      <c r="Z89" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA89" t="n">
         <v>97528</v>
       </c>
-      <c r="Y89" t="n">
+      <c r="AB89" t="n">
         <v>97528</v>
       </c>
-      <c r="Z89" t="n">
+      <c r="AC89" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71779,12 +72586,21 @@
         <v>276400</v>
       </c>
       <c r="X90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y90" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z90" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA90" t="n">
         <v>895000</v>
       </c>
-      <c r="Y90" t="n">
+      <c r="AB90" t="n">
         <v>895000</v>
       </c>
-      <c r="Z90" t="n">
+      <c r="AC90" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71865,12 +72681,21 @@
         <v>0</v>
       </c>
       <c r="X91" t="n">
+        <v>178148.61</v>
+      </c>
+      <c r="Y91" t="n">
+        <v>178148.61</v>
+      </c>
+      <c r="Z91" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA91" t="n">
         <v>86851.39</v>
       </c>
-      <c r="Y91" t="n">
+      <c r="AB91" t="n">
         <v>86851.39</v>
       </c>
-      <c r="Z91" t="n">
+      <c r="AC91" t="n">
         <v>0</v>
       </c>
     </row>
@@ -71951,12 +72776,21 @@
         <v>6000</v>
       </c>
       <c r="X92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y92" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z92" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA92" t="n">
         <v>502286</v>
       </c>
-      <c r="Y92" t="n">
+      <c r="AB92" t="n">
         <v>502286</v>
       </c>
-      <c r="Z92" t="n">
+      <c r="AC92" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72037,12 +72871,21 @@
         <v>0</v>
       </c>
       <c r="X93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y93" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z93" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA93" t="n">
         <v>1312050</v>
       </c>
-      <c r="Y93" t="n">
+      <c r="AB93" t="n">
         <v>1312050</v>
       </c>
-      <c r="Z93" t="n">
+      <c r="AC93" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72126,9 +72969,18 @@
         <v>0</v>
       </c>
       <c r="Y94" t="n">
+        <v>11861411.46</v>
+      </c>
+      <c r="Z94" t="n">
+        <v>11861411.46</v>
+      </c>
+      <c r="AA94" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB94" t="n">
         <v>1824333.68</v>
       </c>
-      <c r="Z94" t="n">
+      <c r="AC94" t="n">
         <v>1824333.68</v>
       </c>
     </row>
@@ -72209,12 +73061,21 @@
         <v>-6636057.49</v>
       </c>
       <c r="X95" t="n">
+        <v>6331411.46</v>
+      </c>
+      <c r="Y95" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z95" t="n">
+        <v>-6331411.46</v>
+      </c>
+      <c r="AA95" t="n">
         <v>7354333.68</v>
       </c>
-      <c r="Y95" t="n">
-        <v>0</v>
-      </c>
-      <c r="Z95" t="n">
+      <c r="AB95" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC95" t="n">
         <v>-7354333.68</v>
       </c>
     </row>
@@ -72295,12 +73156,21 @@
         <v>223121.17</v>
       </c>
       <c r="X96" t="n">
+        <v>415791.82</v>
+      </c>
+      <c r="Y96" t="n">
+        <v>415791.82</v>
+      </c>
+      <c r="Z96" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA96" t="n">
         <v>326945.72</v>
       </c>
-      <c r="Y96" t="n">
+      <c r="AB96" t="n">
         <v>326945.72</v>
       </c>
-      <c r="Z96" t="n">
+      <c r="AC96" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72381,12 +73251,21 @@
         <v>30130.84999999998</v>
       </c>
       <c r="X97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y97" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z97" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA97" t="n">
         <v>1210721.94</v>
       </c>
-      <c r="Y97" t="n">
+      <c r="AB97" t="n">
         <v>1210721.94</v>
       </c>
-      <c r="Z97" t="n">
+      <c r="AC97" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72467,12 +73346,21 @@
         <v>0</v>
       </c>
       <c r="X98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y98" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z98" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA98" t="n">
         <v>100000</v>
       </c>
-      <c r="Y98" t="n">
+      <c r="AB98" t="n">
         <v>100000</v>
       </c>
-      <c r="Z98" t="n">
+      <c r="AC98" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72553,12 +73441,21 @@
         <v>0</v>
       </c>
       <c r="X99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y99" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z99" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA99" t="n">
         <v>490280.12</v>
       </c>
-      <c r="Y99" t="n">
+      <c r="AB99" t="n">
         <v>490280.12</v>
       </c>
-      <c r="Z99" t="n">
+      <c r="AC99" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72639,12 +73536,21 @@
         <v>0</v>
       </c>
       <c r="X100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y100" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z100" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA100" t="n">
         <v>958683.8</v>
       </c>
-      <c r="Y100" t="n">
+      <c r="AB100" t="n">
         <v>958683.8</v>
       </c>
-      <c r="Z100" t="n">
+      <c r="AC100" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72725,12 +73631,21 @@
         <v>0</v>
       </c>
       <c r="X101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y101" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z101" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA101" t="n">
         <v>148969.8</v>
       </c>
-      <c r="Y101" t="n">
+      <c r="AB101" t="n">
         <v>148969.8</v>
       </c>
-      <c r="Z101" t="n">
+      <c r="AC101" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72811,12 +73726,21 @@
         <v>0</v>
       </c>
       <c r="X102" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y102" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z102" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA102" t="n">
         <v>726840.35</v>
       </c>
-      <c r="Y102" t="n">
+      <c r="AB102" t="n">
         <v>726840.35</v>
       </c>
-      <c r="Z102" t="n">
+      <c r="AC102" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72897,12 +73821,21 @@
         <v>0</v>
       </c>
       <c r="X103" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y103" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z103" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA103" t="n">
         <v>1652200</v>
       </c>
-      <c r="Y103" t="n">
+      <c r="AB103" t="n">
         <v>1652200</v>
       </c>
-      <c r="Z103" t="n">
+      <c r="AC103" t="n">
         <v>0</v>
       </c>
     </row>
@@ -72991,6 +73924,15 @@
       <c r="Z104" t="n">
         <v>0</v>
       </c>
+      <c r="AA104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB104" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -73077,6 +74019,15 @@
       <c r="Z105" t="n">
         <v>0</v>
       </c>
+      <c r="AA105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB105" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -73155,12 +74106,21 @@
         <v>0</v>
       </c>
       <c r="X106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y106" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z106" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA106" t="n">
         <v>50000</v>
       </c>
-      <c r="Y106" t="n">
+      <c r="AB106" t="n">
         <v>50000</v>
       </c>
-      <c r="Z106" t="n">
+      <c r="AC106" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73241,12 +74201,21 @@
         <v>0</v>
       </c>
       <c r="X107" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y107" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z107" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA107" t="n">
         <v>249721</v>
       </c>
-      <c r="Y107" t="n">
+      <c r="AB107" t="n">
         <v>249721</v>
       </c>
-      <c r="Z107" t="n">
+      <c r="AC107" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73327,12 +74296,21 @@
         <v>381000</v>
       </c>
       <c r="X108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y108" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z108" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA108" t="n">
         <v>1421600</v>
       </c>
-      <c r="Y108" t="n">
+      <c r="AB108" t="n">
         <v>1414600</v>
       </c>
-      <c r="Z108" t="n">
+      <c r="AC108" t="n">
         <v>-7000</v>
       </c>
     </row>
@@ -73413,12 +74391,21 @@
         <v>0</v>
       </c>
       <c r="X109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y109" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z109" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA109" t="n">
         <v>850000</v>
       </c>
-      <c r="Y109" t="n">
+      <c r="AB109" t="n">
         <v>850000</v>
       </c>
-      <c r="Z109" t="n">
+      <c r="AC109" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73499,12 +74486,21 @@
         <v>929634.22</v>
       </c>
       <c r="X110" t="n">
+        <v>1640638.11</v>
+      </c>
+      <c r="Y110" t="n">
+        <v>1640638.11</v>
+      </c>
+      <c r="Z110" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA110" t="n">
         <v>4429727.67</v>
       </c>
-      <c r="Y110" t="n">
+      <c r="AB110" t="n">
         <v>4429727.67</v>
       </c>
-      <c r="Z110" t="n">
+      <c r="AC110" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73585,12 +74581,21 @@
         <v>0</v>
       </c>
       <c r="X111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y111" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z111" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA111" t="n">
         <v>271067.72</v>
       </c>
-      <c r="Y111" t="n">
+      <c r="AB111" t="n">
         <v>271067.72</v>
       </c>
-      <c r="Z111" t="n">
+      <c r="AC111" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73679,6 +74684,15 @@
       <c r="Z112" t="n">
         <v>0</v>
       </c>
+      <c r="AA112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB112" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -73757,12 +74771,21 @@
         <v>0</v>
       </c>
       <c r="X113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y113" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z113" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA113" t="n">
         <v>308272</v>
       </c>
-      <c r="Y113" t="n">
+      <c r="AB113" t="n">
         <v>308272</v>
       </c>
-      <c r="Z113" t="n">
+      <c r="AC113" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73843,12 +74866,21 @@
         <v>0</v>
       </c>
       <c r="X114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y114" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z114" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA114" t="n">
         <v>1150826</v>
       </c>
-      <c r="Y114" t="n">
+      <c r="AB114" t="n">
         <v>1150826</v>
       </c>
-      <c r="Z114" t="n">
+      <c r="AC114" t="n">
         <v>0</v>
       </c>
     </row>
@@ -73929,12 +74961,21 @@
         <v>0</v>
       </c>
       <c r="X115" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y115" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z115" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA115" t="n">
         <v>2000000</v>
       </c>
-      <c r="Y115" t="n">
+      <c r="AB115" t="n">
         <v>2000000</v>
       </c>
-      <c r="Z115" t="n">
+      <c r="AC115" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74015,12 +75056,21 @@
         <v>0</v>
       </c>
       <c r="X116" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y116" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z116" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA116" t="n">
         <v>29934</v>
       </c>
-      <c r="Y116" t="n">
+      <c r="AB116" t="n">
         <v>29934</v>
       </c>
-      <c r="Z116" t="n">
+      <c r="AC116" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74101,12 +75151,21 @@
         <v>700</v>
       </c>
       <c r="X117" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y117" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z117" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA117" t="n">
         <v>8097000</v>
       </c>
-      <c r="Y117" t="n">
+      <c r="AB117" t="n">
         <v>8097000</v>
       </c>
-      <c r="Z117" t="n">
+      <c r="AC117" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74195,6 +75254,15 @@
       <c r="Z118" t="n">
         <v>0</v>
       </c>
+      <c r="AA118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AB118" t="n">
+        <v>0</v>
+      </c>
+      <c r="AC118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="n">
@@ -74273,12 +75341,21 @@
         <v>0</v>
       </c>
       <c r="X119" t="n">
+        <v>2647578.37</v>
+      </c>
+      <c r="Y119" t="n">
+        <v>2647578.37</v>
+      </c>
+      <c r="Z119" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA119" t="n">
         <v>3627211.32</v>
       </c>
-      <c r="Y119" t="n">
+      <c r="AB119" t="n">
         <v>3627211.32</v>
       </c>
-      <c r="Z119" t="n">
+      <c r="AC119" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74359,12 +75436,21 @@
         <v>0</v>
       </c>
       <c r="X120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y120" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z120" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA120" t="n">
         <v>73000</v>
       </c>
-      <c r="Y120" t="n">
+      <c r="AB120" t="n">
         <v>73000</v>
       </c>
-      <c r="Z120" t="n">
+      <c r="AC120" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74445,12 +75531,21 @@
         <v>371602.3999999999</v>
       </c>
       <c r="X121" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y121" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z121" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA121" t="n">
         <v>2300916.4</v>
       </c>
-      <c r="Y121" t="n">
+      <c r="AB121" t="n">
         <v>2300916.4</v>
       </c>
-      <c r="Z121" t="n">
+      <c r="AC121" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74531,12 +75626,21 @@
         <v>641209.77</v>
       </c>
       <c r="X122" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="Y122" t="n">
+        <v>1000000</v>
+      </c>
+      <c r="Z122" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA122" t="n">
         <v>1076961.03</v>
       </c>
-      <c r="Y122" t="n">
+      <c r="AB122" t="n">
         <v>1076961.03</v>
       </c>
-      <c r="Z122" t="n">
+      <c r="AC122" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74617,12 +75721,21 @@
         <v>0</v>
       </c>
       <c r="X123" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y123" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z123" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA123" t="n">
         <v>180278.9</v>
       </c>
-      <c r="Y123" t="n">
+      <c r="AB123" t="n">
         <v>180278.9</v>
       </c>
-      <c r="Z123" t="n">
+      <c r="AC123" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74703,12 +75816,21 @@
         <v>5550.49</v>
       </c>
       <c r="X124" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y124" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z124" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA124" t="n">
         <v>59848.63</v>
       </c>
-      <c r="Y124" t="n">
+      <c r="AB124" t="n">
         <v>59848.63</v>
       </c>
-      <c r="Z124" t="n">
+      <c r="AC124" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74789,12 +75911,21 @@
         <v>0</v>
       </c>
       <c r="X125" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y125" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z125" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA125" t="n">
         <v>123184.1</v>
       </c>
-      <c r="Y125" t="n">
+      <c r="AB125" t="n">
         <v>123184.1</v>
       </c>
-      <c r="Z125" t="n">
+      <c r="AC125" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74875,12 +76006,21 @@
         <v>0</v>
       </c>
       <c r="X126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y126" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z126" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA126" t="n">
         <v>64000</v>
       </c>
-      <c r="Y126" t="n">
+      <c r="AB126" t="n">
         <v>64000</v>
       </c>
-      <c r="Z126" t="n">
+      <c r="AC126" t="n">
         <v>0</v>
       </c>
     </row>
@@ -74961,12 +76101,21 @@
         <v>0</v>
       </c>
       <c r="X127" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y127" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z127" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA127" t="n">
         <v>10000</v>
       </c>
-      <c r="Y127" t="n">
+      <c r="AB127" t="n">
         <v>10000</v>
       </c>
-      <c r="Z127" t="n">
+      <c r="AC127" t="n">
         <v>0</v>
       </c>
     </row>
@@ -75047,12 +76196,21 @@
         <v>1382898.62</v>
       </c>
       <c r="X128" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="Y128" t="n">
+        <v>15000000</v>
+      </c>
+      <c r="Z128" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA128" t="n">
         <v>10589524.26</v>
       </c>
-      <c r="Y128" t="n">
+      <c r="AB128" t="n">
         <v>10589524.26</v>
       </c>
-      <c r="Z128" t="n">
+      <c r="AC128" t="n">
         <v>0</v>
       </c>
     </row>
@@ -75133,12 +76291,21 @@
         <v>189404.96</v>
       </c>
       <c r="X129" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y129" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z129" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA129" t="n">
         <v>1695593.98</v>
       </c>
-      <c r="Y129" t="n">
+      <c r="AB129" t="n">
         <v>1695593.98</v>
       </c>
-      <c r="Z129" t="n">
+      <c r="AC129" t="n">
         <v>0</v>
       </c>
     </row>
@@ -75219,12 +76386,21 @@
         <v>0</v>
       </c>
       <c r="X130" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y130" t="n">
+        <v>0</v>
+      </c>
+      <c r="Z130" t="n">
+        <v>0</v>
+      </c>
+      <c r="AA130" t="n">
         <v>16394738.95</v>
       </c>
-      <c r="Y130" t="n">
+      <c r="AB130" t="n">
         <v>16272144.64</v>
       </c>
-      <c r="Z130" t="n">
+      <c r="AC130" t="n">
         <v>-122594.3099999987</v>
       </c>
     </row>

</xml_diff>